<commit_message>
Add feature detection analysis and F15 20-view dataset
</commit_message>
<xml_diff>
--- a/feature_detection_analysis/comparison_table.xlsx
+++ b/feature_detection_analysis/comparison_table.xlsx
@@ -529,10 +529,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>299.8417</v>
+        <v>259.9693</v>
       </c>
       <c r="C2" t="n">
-        <v>24.9868</v>
+        <v>12.9985</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -545,34 +545,34 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="G2" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="H2" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="I2" t="n">
         <v>100</v>
       </c>
       <c r="J2" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="K2" t="n">
-        <v>22.73</v>
+        <v>3.57</v>
       </c>
       <c r="L2" t="n">
-        <v>9.09</v>
+        <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>0.088805</v>
+        <v>0.096777</v>
       </c>
       <c r="N2" t="n">
-        <v>2.749506</v>
+        <v>4.366862</v>
       </c>
       <c r="O2" t="n">
-        <v>0.22</v>
+        <v>0.33</v>
       </c>
       <c r="P2" t="n">
         <v>0</v>
@@ -585,49 +585,49 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>703.1462</v>
+        <v>1212.6049</v>
       </c>
       <c r="C3" t="n">
-        <v>58.5955</v>
+        <v>60.6302</v>
       </c>
       <c r="D3" t="n">
-        <v>469.4562</v>
+        <v>1060.8384</v>
       </c>
       <c r="E3" t="n">
-        <v>39.1214</v>
+        <v>53.0419</v>
       </c>
       <c r="F3" t="n">
-        <v>1432</v>
+        <v>2458</v>
       </c>
       <c r="G3" t="n">
-        <v>1432</v>
+        <v>1083</v>
       </c>
       <c r="H3" t="n">
-        <v>924</v>
+        <v>1083</v>
       </c>
       <c r="I3" t="n">
-        <v>64.53</v>
+        <v>100</v>
       </c>
       <c r="J3" t="n">
-        <v>554</v>
+        <v>824</v>
       </c>
       <c r="K3" t="n">
-        <v>40.04</v>
+        <v>23.92</v>
       </c>
       <c r="L3" t="n">
-        <v>18.23</v>
+        <v>21.31</v>
       </c>
       <c r="M3" t="n">
-        <v>0.03531</v>
+        <v>0.032815</v>
       </c>
       <c r="N3" t="n">
-        <v>89.601534</v>
+        <v>113.214935</v>
       </c>
       <c r="O3" t="n">
-        <v>10.8</v>
+        <v>12.84</v>
       </c>
       <c r="P3" t="n">
-        <v>702.11</v>
+        <v>737.0599999999999</v>
       </c>
     </row>
     <row r="4">
@@ -637,10 +637,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.8949</v>
+        <v>4.2902</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3246</v>
+        <v>0.2145</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -653,34 +653,34 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1391</v>
+        <v>4274</v>
       </c>
       <c r="G4" t="n">
-        <v>1391</v>
+        <v>2967</v>
       </c>
       <c r="H4" t="n">
-        <v>930</v>
+        <v>2967</v>
       </c>
       <c r="I4" t="n">
-        <v>66.86</v>
+        <v>100</v>
       </c>
       <c r="J4" t="n">
-        <v>578</v>
+        <v>1652</v>
       </c>
       <c r="K4" t="n">
-        <v>37.85</v>
+        <v>44.32</v>
       </c>
       <c r="L4" t="n">
-        <v>27.98</v>
+        <v>33.85</v>
       </c>
       <c r="M4" t="n">
-        <v>0.025075</v>
+        <v>0.032264</v>
       </c>
       <c r="N4" t="n">
-        <v>93.483189</v>
+        <v>113.214935</v>
       </c>
       <c r="O4" t="n">
-        <v>15.66</v>
+        <v>18.07</v>
       </c>
       <c r="P4" t="n">
         <v>0</v>
@@ -693,10 +693,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>155.3157</v>
+        <v>280.6531</v>
       </c>
       <c r="C5" t="n">
-        <v>12.943</v>
+        <v>14.0327</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -709,34 +709,34 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>558</v>
+        <v>1195</v>
       </c>
       <c r="G5" t="n">
-        <v>558</v>
+        <v>656</v>
       </c>
       <c r="H5" t="n">
-        <v>290</v>
+        <v>656</v>
       </c>
       <c r="I5" t="n">
-        <v>51.97</v>
+        <v>100</v>
       </c>
       <c r="J5" t="n">
-        <v>205</v>
+        <v>406</v>
       </c>
       <c r="K5" t="n">
-        <v>29.31</v>
+        <v>38.11</v>
       </c>
       <c r="L5" t="n">
-        <v>20.95</v>
+        <v>31.86</v>
       </c>
       <c r="M5" t="n">
-        <v>0.042473</v>
+        <v>0.03409</v>
       </c>
       <c r="N5" t="n">
-        <v>33.155802</v>
+        <v>65.66466200000001</v>
       </c>
       <c r="O5" t="n">
-        <v>6.24</v>
+        <v>10.44</v>
       </c>
       <c r="P5" t="n">
         <v>0</v>
@@ -749,49 +749,49 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>310.5204</v>
+        <v>82.1473</v>
       </c>
       <c r="C6" t="n">
-        <v>25.8767</v>
+        <v>4.1074</v>
       </c>
       <c r="D6" t="n">
-        <v>55.7044</v>
+        <v>119.4104</v>
       </c>
       <c r="E6" t="n">
-        <v>4.642</v>
+        <v>5.9705</v>
       </c>
       <c r="F6" t="n">
-        <v>6870</v>
+        <v>11534</v>
       </c>
       <c r="G6" t="n">
-        <v>3000</v>
+        <v>2412</v>
       </c>
       <c r="H6" t="n">
-        <v>1635</v>
+        <v>2412</v>
       </c>
       <c r="I6" t="n">
-        <v>54.5</v>
+        <v>100</v>
       </c>
       <c r="J6" t="n">
-        <v>596</v>
+        <v>1404</v>
       </c>
       <c r="K6" t="n">
-        <v>63.55</v>
+        <v>41.79</v>
       </c>
       <c r="L6" t="n">
-        <v>34.58</v>
+        <v>32.3</v>
       </c>
       <c r="M6" t="n">
-        <v>0.020918</v>
+        <v>0.028935</v>
       </c>
       <c r="N6" t="n">
-        <v>96.39443</v>
+        <v>113.214935</v>
       </c>
       <c r="O6" t="n">
-        <v>10.98</v>
+        <v>14.18</v>
       </c>
       <c r="P6" t="n">
-        <v>702.15</v>
+        <v>738.04</v>
       </c>
     </row>
   </sheetData>

</xml_diff>